<commit_message>
feat(seri-gaya): GB52 rantai — mata rantai terlemah retak, putus, diskor, ditempa ulang (TPRM)
- gb52-rantai: rantai DATAMU→TARIK; satu mata retak (path SVG dash) lalu putus, dokumen berjatuhan;
  tautan asesmen publik + kartu kuesioner ilustrasi; lencana skor per pihak; pijar las; stempel TAHAN
- katalog: 86 video seri gaya SIAP RENDER; sisa TY 1 · GB 39 · PF 26 · SN 11 · UI 17

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/rancangan/Rancangan-Iklan-Video-Privasimu.xlsx
+++ b/rancangan/Rancangan-Iklan-Video-Privasimu.xlsx
@@ -22084,12 +22084,16 @@
           <t>Mata rantai tersambung; satu mata retak.</t>
         </is>
       </c>
-      <c r="E109" s="28" t="inlineStr">
-        <is>
-          <t>Bisa</t>
-        </is>
-      </c>
-      <c r="F109" s="9" t="inlineStr"/>
+      <c r="E109" s="22" t="inlineStr">
+        <is>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="F109" s="9" t="inlineStr">
+        <is>
+          <t>GB52</t>
+        </is>
+      </c>
       <c r="G109" s="9" t="n">
         <v>2</v>
       </c>

</xml_diff>

<commit_message>
feat(seri-gaya): GB40 speedometer — reverse psychology "Jangan lihat jarum ini" (±20 dtk)
- penutup baja "JANGAN LIHAT." + bayangan jarum menari + hitung mundur 3-2-1 → terbelah: jarum berayun lewat 69
  lalu berhenti di 56 CUKUP (antiklimaks) → match-cut ke kartu Privacy Posture Score asli → CTA "Jangan cek skormu.
  Kecuali penasaran."
- sengaja pendek (20,6 dtk): tantangan reverse psychology harus cepat tuntas

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/rancangan/Rancangan-Iklan-Video-Privasimu.xlsx
+++ b/rancangan/Rancangan-Iklan-Video-Privasimu.xlsx
@@ -20660,12 +20660,16 @@
           <t>Jarum meter bergerak dari merah ke hijau.</t>
         </is>
       </c>
-      <c r="E97" s="28" t="inlineStr">
-        <is>
-          <t>Bisa</t>
-        </is>
-      </c>
-      <c r="F97" s="9" t="inlineStr"/>
+      <c r="E97" s="22" t="inlineStr">
+        <is>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="F97" s="9" t="inlineStr">
+        <is>
+          <t>GB40</t>
+        </is>
+      </c>
       <c r="G97" s="9" t="n">
         <v>1</v>
       </c>

</xml_diff>

<commit_message>
feat(seri-gaya): PF32 label museum — "Artefak": spreadsheet & surel berantai dipensiunkan
- aula museum (dunia 3 layar, kamera geser/zoom dari cue), vitrin + lampu sorot + kartu keterangan serif
- twist: kamera mundur, kedua artefak dicap MASIH DIPAKAI*; koleksi terbaru = register RoPA asli
  (kaca terangkat, "sedang dipakai"); penutup mencerminkan bidikan twist: plakat hijau DIPENSIUNKAN ✓
- 9:16: kartu di atas vitrin, judul 56 px

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/rancangan/Rancangan-Iklan-Video-Privasimu.xlsx
+++ b/rancangan/Rancangan-Iklan-Video-Privasimu.xlsx
@@ -35393,12 +35393,16 @@
           <t>Benda di etalase dengan kartu keterangan museum.</t>
         </is>
       </c>
-      <c r="E220" s="28" t="inlineStr">
-        <is>
-          <t>Bisa</t>
-        </is>
-      </c>
-      <c r="F220" s="19" t="inlineStr"/>
+      <c r="E220" s="22" t="inlineStr">
+        <is>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="F220" s="19" t="inlineStr">
+        <is>
+          <t>PF32</t>
+        </is>
+      </c>
       <c r="G220" s="19" t="n">
         <v>2</v>
       </c>

</xml_diff>